<commit_message>
journal 31.07 till september
</commit_message>
<xml_diff>
--- a/ჟურნალი/6. N301 front-end ხელოვნური ინტელექტის გამოყენება.xlsx
+++ b/ჟურნალი/6. N301 front-end ხელოვნური ინტელექტის გამოყენება.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3Daudiece\Desktop\Front-end!!\0. ready\ჟურნალი\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB720129-2995-413B-91F0-A340F691B923}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297460EE-145F-412A-A8BC-30FA6DC9DE08}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-122" yWindow="-122" windowWidth="29045" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="51">
   <si>
     <t xml:space="preserve">პროგრამა                     </t>
   </si>
@@ -504,7 +504,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -532,6 +532,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -692,7 +698,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -832,6 +838,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1257,7 +1269,7 @@
       <c r="AF2" s="29">
         <v>46232</v>
       </c>
-      <c r="AG2" s="29">
+      <c r="AG2" s="52">
         <v>46234</v>
       </c>
       <c r="AH2" s="29"/>
@@ -1337,7 +1349,7 @@
       <c r="AD3" s="29"/>
       <c r="AE3" s="29"/>
       <c r="AF3" s="29"/>
-      <c r="AG3" s="29"/>
+      <c r="AG3" s="52"/>
       <c r="AH3" s="29"/>
       <c r="AI3" s="29"/>
       <c r="AJ3" s="29"/>
@@ -1417,7 +1429,7 @@
       <c r="AD4" s="29"/>
       <c r="AE4" s="29"/>
       <c r="AF4" s="29"/>
-      <c r="AG4" s="29"/>
+      <c r="AG4" s="52"/>
       <c r="AH4" s="29"/>
       <c r="AI4" s="29"/>
       <c r="AJ4" s="29"/>
@@ -1497,7 +1509,7 @@
       <c r="AD5" s="29"/>
       <c r="AE5" s="29"/>
       <c r="AF5" s="29"/>
-      <c r="AG5" s="29"/>
+      <c r="AG5" s="52"/>
       <c r="AH5" s="29"/>
       <c r="AI5" s="29"/>
       <c r="AJ5" s="29"/>
@@ -1577,7 +1589,7 @@
       <c r="AD6" s="29"/>
       <c r="AE6" s="29"/>
       <c r="AF6" s="29"/>
-      <c r="AG6" s="29"/>
+      <c r="AG6" s="52"/>
       <c r="AH6" s="29"/>
       <c r="AI6" s="29"/>
       <c r="AJ6" s="29"/>
@@ -1657,7 +1669,7 @@
       <c r="AD7" s="30"/>
       <c r="AE7" s="30"/>
       <c r="AF7" s="30"/>
-      <c r="AG7" s="30"/>
+      <c r="AG7" s="53"/>
       <c r="AH7" s="30"/>
       <c r="AI7" s="30"/>
       <c r="AJ7" s="30"/>
@@ -2231,7 +2243,7 @@
       </c>
       <c r="D11" s="11">
         <f t="shared" ref="D11:D28" si="0">COUNT(F11:BV11)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="8"/>
@@ -2271,7 +2283,9 @@
       <c r="AF11" s="8">
         <v>0</v>
       </c>
-      <c r="AG11" s="8"/>
+      <c r="AG11" s="8">
+        <v>0</v>
+      </c>
       <c r="AH11" s="8"/>
       <c r="AI11" s="8"/>
       <c r="AJ11" s="8"/>
@@ -2411,7 +2425,7 @@
       </c>
       <c r="D13" s="11">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="8"/>
@@ -2465,7 +2479,9 @@
       <c r="AF13" s="8">
         <v>0</v>
       </c>
-      <c r="AG13" s="8"/>
+      <c r="AG13" s="8">
+        <v>0</v>
+      </c>
       <c r="AH13" s="8"/>
       <c r="AI13" s="8"/>
       <c r="AJ13" s="8"/>
@@ -2524,7 +2540,7 @@
       </c>
       <c r="D14" s="11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" s="12"/>
       <c r="F14" s="8"/>
@@ -2572,7 +2588,9 @@
       <c r="AF14" s="8">
         <v>0</v>
       </c>
-      <c r="AG14" s="8"/>
+      <c r="AG14" s="8">
+        <v>0</v>
+      </c>
       <c r="AH14" s="8"/>
       <c r="AI14" s="8"/>
       <c r="AJ14" s="8"/>
@@ -2627,7 +2645,7 @@
       </c>
       <c r="D15" s="11">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="8">
@@ -2683,7 +2701,9 @@
       <c r="AF15" s="8">
         <v>0</v>
       </c>
-      <c r="AG15" s="8"/>
+      <c r="AG15" s="8">
+        <v>0</v>
+      </c>
       <c r="AH15" s="8"/>
       <c r="AI15" s="8"/>
       <c r="AJ15" s="8"/>
@@ -2738,7 +2758,7 @@
       </c>
       <c r="D16" s="11">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="8"/>
@@ -2780,7 +2800,9 @@
       <c r="AF16" s="8">
         <v>0</v>
       </c>
-      <c r="AG16" s="8"/>
+      <c r="AG16" s="8">
+        <v>0</v>
+      </c>
       <c r="AH16" s="8"/>
       <c r="AI16" s="8"/>
       <c r="AJ16" s="8"/>
@@ -2934,7 +2956,7 @@
       </c>
       <c r="D18" s="11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="8">
@@ -2982,7 +3004,9 @@
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
       <c r="AF18" s="8"/>
-      <c r="AG18" s="8"/>
+      <c r="AG18" s="8">
+        <v>0</v>
+      </c>
       <c r="AH18" s="8"/>
       <c r="AI18" s="8"/>
       <c r="AJ18" s="8"/>
@@ -3245,7 +3269,7 @@
       </c>
       <c r="D21" s="11">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="8">
@@ -3329,7 +3353,9 @@
       <c r="AF21" s="8">
         <v>0</v>
       </c>
-      <c r="AG21" s="8"/>
+      <c r="AG21" s="8">
+        <v>0</v>
+      </c>
       <c r="AH21" s="8"/>
       <c r="AI21" s="8"/>
       <c r="AJ21" s="8"/>
@@ -3384,7 +3410,7 @@
       </c>
       <c r="D22" s="11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E22" s="12"/>
       <c r="F22" s="8"/>
@@ -3432,7 +3458,9 @@
       <c r="AF22" s="8">
         <v>0</v>
       </c>
-      <c r="AG22" s="8"/>
+      <c r="AG22" s="8">
+        <v>0</v>
+      </c>
       <c r="AH22" s="8"/>
       <c r="AI22" s="8"/>
       <c r="AJ22" s="8"/>
@@ -3487,7 +3515,7 @@
       </c>
       <c r="D23" s="11">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E23" s="12"/>
       <c r="F23" s="8">
@@ -3571,7 +3599,9 @@
       <c r="AF23" s="8">
         <v>0</v>
       </c>
-      <c r="AG23" s="8"/>
+      <c r="AG23" s="8">
+        <v>0</v>
+      </c>
       <c r="AH23" s="8"/>
       <c r="AI23" s="8"/>
       <c r="AJ23" s="8"/>
@@ -3626,7 +3656,7 @@
       </c>
       <c r="D24" s="11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" s="12"/>
       <c r="F24" s="8">
@@ -3674,7 +3704,9 @@
       <c r="AF24" s="8">
         <v>0</v>
       </c>
-      <c r="AG24" s="8"/>
+      <c r="AG24" s="8">
+        <v>0</v>
+      </c>
       <c r="AH24" s="8"/>
       <c r="AI24" s="8"/>
       <c r="AJ24" s="8"/>
@@ -3729,7 +3761,7 @@
       </c>
       <c r="D25" s="11">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E25" s="12"/>
       <c r="F25" s="8">
@@ -3785,7 +3817,9 @@
       <c r="AF25" s="8">
         <v>0</v>
       </c>
-      <c r="AG25" s="8"/>
+      <c r="AG25" s="8">
+        <v>0</v>
+      </c>
       <c r="AH25" s="8"/>
       <c r="AI25" s="8"/>
       <c r="AJ25" s="8"/>
@@ -3840,7 +3874,7 @@
       </c>
       <c r="D26" s="11">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" s="12"/>
       <c r="F26" s="8">
@@ -3896,7 +3930,9 @@
       <c r="AF26" s="8">
         <v>0</v>
       </c>
-      <c r="AG26" s="8"/>
+      <c r="AG26" s="8">
+        <v>0</v>
+      </c>
       <c r="AH26" s="8"/>
       <c r="AI26" s="8"/>
       <c r="AJ26" s="8"/>
@@ -3951,7 +3987,7 @@
       </c>
       <c r="D27" s="11">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E27" s="15"/>
       <c r="F27" s="8">
@@ -4035,7 +4071,9 @@
       <c r="AF27" s="8">
         <v>0</v>
       </c>
-      <c r="AG27" s="8"/>
+      <c r="AG27" s="8">
+        <v>0</v>
+      </c>
       <c r="AH27" s="8"/>
       <c r="AI27" s="8"/>
       <c r="AJ27" s="8"/>

</xml_diff>